<commit_message>
Update Trading Journal.xlsx 2026-08-19 07:36:07
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -612,6 +612,35 @@
         <v>1</v>
       </c>
       <c r="G6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>1233</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-19 07:42:57
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -425,7 +425,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -614,11 +614,7 @@
       <c r="G6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
+      <c r="A7" s="1" t="inlineStr"/>
       <c r="B7" s="1" t="inlineStr">
         <is>
           <t>1303</t>
@@ -629,17 +625,9 @@
           <t>南亞</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>1233</v>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>3K反轉</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>1</v>
-      </c>
+      <c r="D7" s="1" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-22 09:45:01
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -423,8 +423,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -614,19 +614,29 @@
       <c r="G6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>00404A</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>南亞</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr"/>
+          <t>主動聯博動能50</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>反向島狀</t>
+        </is>
+      </c>
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-22 10:00:11
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,8 +637,39 @@
           <t>反向島狀</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="G7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>00404A</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>主動聯博動能50</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-22 10:13:12
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -670,6 +670,33 @@
         <v>1</v>
       </c>
       <c r="G8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>00407A</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>主動凱基台灣</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>222</v>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-22 10:41:20
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -616,87 +616,29 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>00404A</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>主動聯博動能50</t>
+          <t>大立光</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>111</v>
+        <v>4444</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>反向島狀</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>1</v>
-      </c>
+          <t>停利賣出</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>00404A</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>主動聯博動能50</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>111</v>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>停利賣出</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="1" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>00407A</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>主動凱基台灣</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>222</v>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>停利賣出</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr"/>
-      <c r="G9" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 22:52:37
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -429,6 +429,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,15 +455,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>買賣方向</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>進出手法</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>買賣張數</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -489,13 +495,18 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
           <t>島狀反轉</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -518,13 +529,18 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="G3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -547,13 +563,18 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
           <t>島狀反轉</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -576,13 +597,18 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
           <t>KD高腳</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="G5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -605,13 +631,18 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
           <t>3K反轉</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="G6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -634,11 +665,48 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
           <t>停利賣出</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 22:55:36
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -675,38 +675,6 @@
       </c>
       <c r="G7" s="1" t="inlineStr"/>
       <c r="H7" s="1" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>3605</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>宏致</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>107</v>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>巧妙點</t>
-        </is>
-      </c>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 22:59:54
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -643,38 +643,6 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>3008</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>大立光</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>4444</v>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>賣出</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>停利賣出</t>
-        </is>
-      </c>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 23:12:00
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -609,40 +609,6 @@
         <v>2</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>2645</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>長榮航太</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>193.5</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>3K反轉</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 23:12:41
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -609,6 +609,40 @@
         <v>2</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>2615</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>萬海</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-08-28 23:37:54
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -477,21 +477,21 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>8261</t>
+          <t>2615</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>富鼎</t>
+          <t>萬海</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>173</v>
+        <v>113</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
@@ -500,149 +500,13 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>島狀反轉</t>
+          <t>巧妙點</t>
         </is>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>8261</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>富鼎</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>248</v>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>賣出</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>停利賣出</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>5483</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>中美晶</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>192</v>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>島狀反轉</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="1" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>4566</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>時碩工業</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>79</v>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>KD高腳</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>2615</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>萬海</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>113</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>巧妙點</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-06 23:05:18
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -507,6 +507,40 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-06 23:08:49
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -541,6 +541,40 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>3605</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>宏致</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>跌停</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-06 23:23:49
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -575,6 +575,38 @@
         <v>1</v>
       </c>
       <c r="H4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>3441</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>聯一光</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-08 23:06:43
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,36 @@
       </c>
       <c r="G5" s="1" t="inlineStr"/>
       <c r="H5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>2303</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>聯電</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-08 23:44:03
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -579,64 +579,32 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>3441</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>聯一光</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>130</v>
+        <v>137.5</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>3K反轉</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="H5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>2303</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>聯電</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>137.5</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-08 23:48:18
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,12 +419,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -605,6 +605,38 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>00408A</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>主動第一金優股息</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>反向島狀</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-08 23:51:47
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,38 @@
       </c>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>00407A</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>主動凱基台灣</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>反向島狀</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 00:00:19
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,6 +669,34 @@
       </c>
       <c r="G7" s="1" t="inlineStr"/>
       <c r="H7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>00406A</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>主動中信台灣收益</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 00:07:01
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -609,94 +609,30 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>00408A</t>
+          <t>00406A</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>主動第一金優股息</t>
+          <t>主動中信台灣收益</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>111</v>
+        <v>11</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>反向島狀</t>
-        </is>
-      </c>
+      <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>00407A</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>主動凱基台灣</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>反向島狀</t>
-        </is>
-      </c>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>00406A</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>主動中信台灣收益</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr"/>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 10:04:23
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,12 +419,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -605,34 +605,6 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>00406A</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>主動中信台灣收益</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 10:07:49
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -605,6 +605,34 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>8064</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>東捷</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 10:53:58
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -605,34 +605,6 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>8064</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>東捷</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 10:56:13
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,12 +419,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -605,6 +605,34 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>00406A</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>主動中信台灣收益</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 22:51:48
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -600,7 +600,11 @@
           <t>買入</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>單跳空</t>
+        </is>
+      </c>
       <c r="G5" s="1" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-09 22:56:07
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,34 @@
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>4958</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>臻鼎-KY</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>506</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr"/>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>